<commit_message>
upgrades: Removing unnecessary libs to lighten project
</commit_message>
<xml_diff>
--- a/ressources/GPROJ/Tasks.xlsx
+++ b/ressources/GPROJ/Tasks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Félisme\Documents\Vector Software Analyzer\vector_software\ressources\GPROJ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{183E2B39-6E31-42C6-9118-CF2472BDC33D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAEED8DF-C714-44F2-BF3E-FDDF75C1AB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="51">
   <si>
     <t>Bug</t>
   </si>
@@ -76,6 +76,135 @@
   </si>
   <si>
     <t>Date</t>
+  </si>
+  <si>
+    <t>Build trop lourde</t>
+  </si>
+  <si>
+    <t>Changer les imports
+Remplacer sklearn par numpy</t>
+  </si>
+  <si>
+    <t>TODO</t>
+  </si>
+  <si>
+    <t>Upgrades</t>
+  </si>
+  <si>
+    <t>Splash Screen</t>
+  </si>
+  <si>
+    <t>Vertical Wind</t>
+  </si>
+  <si>
+    <t>Fenêtre à part pour visualiser
+le vent vertical sur skew-T</t>
+  </si>
+  <si>
+    <t>Permet de comprendre
+ quand le logiciel est lancé</t>
+  </si>
+  <si>
+    <t>Curseur 
+Skew T</t>
+  </si>
+  <si>
+    <t>Epurer le curseur pour
+affiché seulement les 
+courbes interessantes</t>
+  </si>
+  <si>
+    <t>Export 
+Preferences</t>
+  </si>
+  <si>
+    <t>Permet de changer 
+les paramètres d'export
+pour kml</t>
+  </si>
+  <si>
+    <t>Menu Version</t>
+  </si>
+  <si>
+    <t>Permet de checker
+si logiciel à jour
+et télécharger si il faut</t>
+  </si>
+  <si>
+    <t>Manuel</t>
+  </si>
+  <si>
+    <t>Faire manuel</t>
+  </si>
+  <si>
+    <t>Compatibilité</t>
+  </si>
+  <si>
+    <t>Faire en sorte
+que ce soit 
+compatible Mac</t>
+  </si>
+  <si>
+    <t>Cross visualization</t>
+  </si>
+  <si>
+    <t>Permet de 
+sélectionner un 
+point et de le voir
+dans chaque tab</t>
+  </si>
+  <si>
+    <t>Refonte</t>
+  </si>
+  <si>
+    <t>Refonte du 
+code entier
+avec classe</t>
+  </si>
+  <si>
+    <t>Documenter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documenter correctement </t>
+  </si>
+  <si>
+    <t>Dark Mode</t>
+  </si>
+  <si>
+    <t>Langages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Changer automatique
+le langage </t>
+  </si>
+  <si>
+    <t>Changement d'unité 
+non appliqué sur variable 
+1D</t>
+  </si>
+  <si>
+    <t>Dynamic Tab</t>
+  </si>
+  <si>
+    <t>Ajouter le tab Dynamic</t>
+  </si>
+  <si>
+    <t>Preference Tiles</t>
+  </si>
+  <si>
+    <t>Pouvoir choisir sa
+source de tuiles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read IGC </t>
+  </si>
+  <si>
+    <t>Alti ground</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Récupérer topo
+et calculer l'alti
+au sol </t>
   </si>
 </sst>
 </file>
@@ -91,7 +220,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -107,6 +236,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -138,12 +273,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,9 +564,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="D9:V37"/>
+  <dimension ref="D7:AG37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="4" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.109375" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" customWidth="1"/>
     <col min="8" max="8" width="12.21875" customWidth="1"/>
@@ -434,15 +575,28 @@
     <col min="10" max="10" width="16.44140625" customWidth="1"/>
     <col min="11" max="11" width="15.109375" customWidth="1"/>
     <col min="12" max="13" width="32.77734375" customWidth="1"/>
+    <col min="14" max="14" width="10.77734375" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="13.21875" customWidth="1"/>
     <col min="16" max="16" width="15.33203125" customWidth="1"/>
     <col min="17" max="17" width="13.109375" customWidth="1"/>
     <col min="19" max="19" width="14.88671875" customWidth="1"/>
     <col min="20" max="20" width="13.77734375" customWidth="1"/>
     <col min="21" max="22" width="13.33203125" customWidth="1"/>
+    <col min="25" max="25" width="13.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="9" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="7" spans="4:33" x14ac:dyDescent="0.3">
+      <c r="D7" t="s">
+        <v>0</v>
+      </c>
+      <c r="N7" t="s">
+        <v>5</v>
+      </c>
+      <c r="Y7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D9" s="2" t="s">
         <v>14</v>
       </c>
@@ -498,28 +652,92 @@
       <c r="V9" s="3" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="10" spans="4:22" x14ac:dyDescent="0.3">
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="Y9" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="Z9" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="AA9" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AB9" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="AC9" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="AD9" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AE9" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="AF9" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="AG9" s="7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="4:33" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="D10" s="5">
+        <v>46149</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>43</v>
+      </c>
       <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
+      <c r="G10" s="1">
+        <v>3</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
-      <c r="N10" s="1"/>
-      <c r="O10" s="1"/>
-      <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
-      <c r="R10" s="1"/>
+      <c r="N10" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P10" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q10" s="1">
+        <v>3</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
       <c r="U10" s="1"/>
       <c r="V10" s="1"/>
-    </row>
-    <row r="11" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y10" s="5">
+        <v>46149</v>
+      </c>
+      <c r="Z10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="AA10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB10" s="1">
+        <v>4</v>
+      </c>
+      <c r="AC10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD10" s="1"/>
+      <c r="AE10" s="1"/>
+      <c r="AF10" s="1"/>
+      <c r="AG10" s="1"/>
+    </row>
+    <row r="11" spans="4:33" ht="129.6" x14ac:dyDescent="0.3">
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
@@ -530,17 +748,46 @@
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
       <c r="M11" s="4"/>
-      <c r="N11" s="1"/>
-      <c r="O11" s="1"/>
-      <c r="P11" s="1"/>
-      <c r="Q11" s="1"/>
-      <c r="R11" s="1"/>
+      <c r="N11" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="P11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q11" s="1">
+        <v>2</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
       <c r="U11" s="1"/>
       <c r="V11" s="1"/>
-    </row>
-    <row r="12" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y11" s="5">
+        <v>46149</v>
+      </c>
+      <c r="Z11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="AA11" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="AB11" s="1">
+        <v>2</v>
+      </c>
+      <c r="AC11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD11" s="1"/>
+      <c r="AE11" s="1"/>
+      <c r="AF11" s="1"/>
+      <c r="AG11" s="1"/>
+    </row>
+    <row r="12" spans="4:33" ht="86.4" x14ac:dyDescent="0.3">
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
@@ -551,17 +798,46 @@
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
       <c r="M12" s="4"/>
-      <c r="N12" s="1"/>
-      <c r="O12" s="1"/>
-      <c r="P12" s="1"/>
-      <c r="Q12" s="1"/>
-      <c r="R12" s="1"/>
+      <c r="N12" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O12" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="P12" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q12" s="1">
+        <v>2</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
-    </row>
-    <row r="13" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y12" s="5">
+        <v>46149</v>
+      </c>
+      <c r="Z12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AA12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="AB12" s="1">
+        <v>4</v>
+      </c>
+      <c r="AC12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD12" s="1"/>
+      <c r="AE12" s="1"/>
+      <c r="AF12" s="1"/>
+      <c r="AG12" s="1"/>
+    </row>
+    <row r="13" spans="4:33" ht="86.4" x14ac:dyDescent="0.3">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -572,17 +848,46 @@
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
       <c r="M13" s="4"/>
-      <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
-      <c r="P13" s="1"/>
-      <c r="Q13" s="1"/>
-      <c r="R13" s="1"/>
+      <c r="N13" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="P13" s="6" t="s">
+        <v>29</v>
+      </c>
+      <c r="Q13" s="1">
+        <v>2</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
-    </row>
-    <row r="14" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y13" s="5">
+        <v>46149</v>
+      </c>
+      <c r="Z13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="AA13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="AB13" s="1">
+        <v>4</v>
+      </c>
+      <c r="AC13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD13" s="1"/>
+      <c r="AE13" s="1"/>
+      <c r="AF13" s="1"/>
+      <c r="AG13" s="1"/>
+    </row>
+    <row r="14" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
@@ -593,17 +898,46 @@
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
       <c r="M14" s="4"/>
-      <c r="N14" s="1"/>
-      <c r="O14" s="1"/>
-      <c r="P14" s="1"/>
-      <c r="Q14" s="1"/>
-      <c r="R14" s="1"/>
+      <c r="N14" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="Q14" s="1">
+        <v>3</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
-    </row>
-    <row r="15" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y14" s="5">
+        <v>46149</v>
+      </c>
+      <c r="Z14" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="AA14" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="AB14" s="1">
+        <v>4</v>
+      </c>
+      <c r="AC14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="AD14" s="1"/>
+      <c r="AE14" s="1"/>
+      <c r="AF14" s="1"/>
+      <c r="AG14" s="1"/>
+    </row>
+    <row r="15" spans="4:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
@@ -614,17 +948,36 @@
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
       <c r="M15" s="4"/>
-      <c r="N15" s="1"/>
-      <c r="O15" s="1"/>
-      <c r="P15" s="1"/>
-      <c r="Q15" s="1"/>
-      <c r="R15" s="1"/>
+      <c r="N15" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="P15" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q15" s="1">
+        <v>1</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
-    </row>
-    <row r="16" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y15" s="1"/>
+      <c r="Z15" s="1"/>
+      <c r="AA15" s="1"/>
+      <c r="AB15" s="1"/>
+      <c r="AC15" s="1"/>
+      <c r="AD15" s="1"/>
+      <c r="AE15" s="1"/>
+      <c r="AF15" s="1"/>
+      <c r="AG15" s="1"/>
+    </row>
+    <row r="16" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
@@ -635,17 +988,34 @@
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
       <c r="M16" s="4"/>
-      <c r="N16" s="1"/>
-      <c r="O16" s="1"/>
+      <c r="N16" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="P16" s="1"/>
-      <c r="Q16" s="1"/>
-      <c r="R16" s="1"/>
+      <c r="Q16" s="1">
+        <v>1</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
-    </row>
-    <row r="17" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y16" s="1"/>
+      <c r="Z16" s="1"/>
+      <c r="AA16" s="1"/>
+      <c r="AB16" s="1"/>
+      <c r="AC16" s="1"/>
+      <c r="AD16" s="1"/>
+      <c r="AE16" s="1"/>
+      <c r="AF16" s="1"/>
+      <c r="AG16" s="1"/>
+    </row>
+    <row r="17" spans="4:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
@@ -656,17 +1026,36 @@
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="4"/>
-      <c r="N17" s="1"/>
-      <c r="O17" s="1"/>
-      <c r="P17" s="1"/>
-      <c r="Q17" s="1"/>
-      <c r="R17" s="1"/>
+      <c r="N17" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O17" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P17" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q17" s="1">
+        <v>2</v>
+      </c>
+      <c r="R17" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
-    </row>
-    <row r="18" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y17" s="1"/>
+      <c r="Z17" s="1"/>
+      <c r="AA17" s="1"/>
+      <c r="AB17" s="1"/>
+      <c r="AC17" s="1"/>
+      <c r="AD17" s="1"/>
+      <c r="AE17" s="1"/>
+      <c r="AF17" s="1"/>
+      <c r="AG17" s="1"/>
+    </row>
+    <row r="18" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
@@ -677,17 +1066,36 @@
       <c r="K18" s="1"/>
       <c r="L18" s="1"/>
       <c r="M18" s="4"/>
-      <c r="N18" s="1"/>
-      <c r="O18" s="1"/>
-      <c r="P18" s="1"/>
-      <c r="Q18" s="1"/>
-      <c r="R18" s="1"/>
+      <c r="N18" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O18" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="P18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q18" s="1">
+        <v>4</v>
+      </c>
+      <c r="R18" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S18" s="1"/>
       <c r="T18" s="1"/>
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
-    </row>
-    <row r="19" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y18" s="1"/>
+      <c r="Z18" s="1"/>
+      <c r="AA18" s="1"/>
+      <c r="AB18" s="1"/>
+      <c r="AC18" s="1"/>
+      <c r="AD18" s="1"/>
+      <c r="AE18" s="1"/>
+      <c r="AF18" s="1"/>
+      <c r="AG18" s="1"/>
+    </row>
+    <row r="19" spans="4:33" ht="28.8" x14ac:dyDescent="0.3">
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
@@ -698,17 +1106,36 @@
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
       <c r="M19" s="4"/>
-      <c r="N19" s="1"/>
-      <c r="O19" s="1"/>
-      <c r="P19" s="1"/>
-      <c r="Q19" s="1"/>
-      <c r="R19" s="1"/>
+      <c r="N19" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="P19" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q19" s="1">
+        <v>2</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
-    </row>
-    <row r="20" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y19" s="1"/>
+      <c r="Z19" s="1"/>
+      <c r="AA19" s="1"/>
+      <c r="AB19" s="1"/>
+      <c r="AC19" s="1"/>
+      <c r="AD19" s="1"/>
+      <c r="AE19" s="1"/>
+      <c r="AF19" s="1"/>
+      <c r="AG19" s="1"/>
+    </row>
+    <row r="20" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
@@ -719,17 +1146,34 @@
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="4"/>
-      <c r="N20" s="1"/>
-      <c r="O20" s="1"/>
+      <c r="N20" s="5">
+        <v>45784</v>
+      </c>
+      <c r="O20" s="1" t="s">
+        <v>48</v>
+      </c>
       <c r="P20" s="1"/>
-      <c r="Q20" s="1"/>
-      <c r="R20" s="1"/>
+      <c r="Q20" s="1">
+        <v>1</v>
+      </c>
+      <c r="R20" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
-    </row>
-    <row r="21" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y20" s="1"/>
+      <c r="Z20" s="1"/>
+      <c r="AA20" s="1"/>
+      <c r="AB20" s="1"/>
+      <c r="AC20" s="1"/>
+      <c r="AD20" s="1"/>
+      <c r="AE20" s="1"/>
+      <c r="AF20" s="1"/>
+      <c r="AG20" s="1"/>
+    </row>
+    <row r="21" spans="4:33" ht="43.2" x14ac:dyDescent="0.3">
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
@@ -740,17 +1184,36 @@
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
       <c r="M21" s="4"/>
-      <c r="N21" s="1"/>
-      <c r="O21" s="1"/>
-      <c r="P21" s="1"/>
-      <c r="Q21" s="1"/>
-      <c r="R21" s="1"/>
+      <c r="N21" s="5">
+        <v>45785</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="P21" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="Q21" s="1">
+        <v>2</v>
+      </c>
+      <c r="R21" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
-    </row>
-    <row r="22" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y21" s="1"/>
+      <c r="Z21" s="1"/>
+      <c r="AA21" s="1"/>
+      <c r="AB21" s="1"/>
+      <c r="AC21" s="1"/>
+      <c r="AD21" s="1"/>
+      <c r="AE21" s="1"/>
+      <c r="AF21" s="1"/>
+      <c r="AG21" s="1"/>
+    </row>
+    <row r="22" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
@@ -770,8 +1233,17 @@
       <c r="T22" s="1"/>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
-    </row>
-    <row r="23" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y22" s="1"/>
+      <c r="Z22" s="1"/>
+      <c r="AA22" s="1"/>
+      <c r="AB22" s="1"/>
+      <c r="AC22" s="1"/>
+      <c r="AD22" s="1"/>
+      <c r="AE22" s="1"/>
+      <c r="AF22" s="1"/>
+      <c r="AG22" s="1"/>
+    </row>
+    <row r="23" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
@@ -791,8 +1263,17 @@
       <c r="T23" s="1"/>
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
-    </row>
-    <row r="24" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y23" s="1"/>
+      <c r="Z23" s="1"/>
+      <c r="AA23" s="1"/>
+      <c r="AB23" s="1"/>
+      <c r="AC23" s="1"/>
+      <c r="AD23" s="1"/>
+      <c r="AE23" s="1"/>
+      <c r="AF23" s="1"/>
+      <c r="AG23" s="1"/>
+    </row>
+    <row r="24" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
@@ -812,8 +1293,17 @@
       <c r="T24" s="1"/>
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
-    </row>
-    <row r="25" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y24" s="1"/>
+      <c r="Z24" s="1"/>
+      <c r="AA24" s="1"/>
+      <c r="AB24" s="1"/>
+      <c r="AC24" s="1"/>
+      <c r="AD24" s="1"/>
+      <c r="AE24" s="1"/>
+      <c r="AF24" s="1"/>
+      <c r="AG24" s="1"/>
+    </row>
+    <row r="25" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
@@ -833,8 +1323,17 @@
       <c r="T25" s="1"/>
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
-    </row>
-    <row r="26" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y25" s="1"/>
+      <c r="Z25" s="1"/>
+      <c r="AA25" s="1"/>
+      <c r="AB25" s="1"/>
+      <c r="AC25" s="1"/>
+      <c r="AD25" s="1"/>
+      <c r="AE25" s="1"/>
+      <c r="AF25" s="1"/>
+      <c r="AG25" s="1"/>
+    </row>
+    <row r="26" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
@@ -854,8 +1353,17 @@
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
-    </row>
-    <row r="27" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y26" s="1"/>
+      <c r="Z26" s="1"/>
+      <c r="AA26" s="1"/>
+      <c r="AB26" s="1"/>
+      <c r="AC26" s="1"/>
+      <c r="AD26" s="1"/>
+      <c r="AE26" s="1"/>
+      <c r="AF26" s="1"/>
+      <c r="AG26" s="1"/>
+    </row>
+    <row r="27" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
@@ -875,8 +1383,17 @@
       <c r="T27" s="1"/>
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
-    </row>
-    <row r="28" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y27" s="1"/>
+      <c r="Z27" s="1"/>
+      <c r="AA27" s="1"/>
+      <c r="AB27" s="1"/>
+      <c r="AC27" s="1"/>
+      <c r="AD27" s="1"/>
+      <c r="AE27" s="1"/>
+      <c r="AF27" s="1"/>
+      <c r="AG27" s="1"/>
+    </row>
+    <row r="28" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
@@ -896,8 +1413,17 @@
       <c r="T28" s="1"/>
       <c r="U28" s="1"/>
       <c r="V28" s="1"/>
-    </row>
-    <row r="29" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y28" s="1"/>
+      <c r="Z28" s="1"/>
+      <c r="AA28" s="1"/>
+      <c r="AB28" s="1"/>
+      <c r="AC28" s="1"/>
+      <c r="AD28" s="1"/>
+      <c r="AE28" s="1"/>
+      <c r="AF28" s="1"/>
+      <c r="AG28" s="1"/>
+    </row>
+    <row r="29" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
@@ -917,8 +1443,17 @@
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
-    </row>
-    <row r="30" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y29" s="1"/>
+      <c r="Z29" s="1"/>
+      <c r="AA29" s="1"/>
+      <c r="AB29" s="1"/>
+      <c r="AC29" s="1"/>
+      <c r="AD29" s="1"/>
+      <c r="AE29" s="1"/>
+      <c r="AF29" s="1"/>
+      <c r="AG29" s="1"/>
+    </row>
+    <row r="30" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
@@ -938,8 +1473,17 @@
       <c r="T30" s="1"/>
       <c r="U30" s="1"/>
       <c r="V30" s="1"/>
-    </row>
-    <row r="31" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y30" s="1"/>
+      <c r="Z30" s="1"/>
+      <c r="AA30" s="1"/>
+      <c r="AB30" s="1"/>
+      <c r="AC30" s="1"/>
+      <c r="AD30" s="1"/>
+      <c r="AE30" s="1"/>
+      <c r="AF30" s="1"/>
+      <c r="AG30" s="1"/>
+    </row>
+    <row r="31" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D31" s="1"/>
       <c r="E31" s="1"/>
       <c r="F31" s="1"/>
@@ -959,8 +1503,17 @@
       <c r="T31" s="1"/>
       <c r="U31" s="1"/>
       <c r="V31" s="1"/>
-    </row>
-    <row r="32" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y31" s="1"/>
+      <c r="Z31" s="1"/>
+      <c r="AA31" s="1"/>
+      <c r="AB31" s="1"/>
+      <c r="AC31" s="1"/>
+      <c r="AD31" s="1"/>
+      <c r="AE31" s="1"/>
+      <c r="AF31" s="1"/>
+      <c r="AG31" s="1"/>
+    </row>
+    <row r="32" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D32" s="1"/>
       <c r="E32" s="1"/>
       <c r="F32" s="1"/>
@@ -980,8 +1533,17 @@
       <c r="T32" s="1"/>
       <c r="U32" s="1"/>
       <c r="V32" s="1"/>
-    </row>
-    <row r="33" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y32" s="1"/>
+      <c r="Z32" s="1"/>
+      <c r="AA32" s="1"/>
+      <c r="AB32" s="1"/>
+      <c r="AC32" s="1"/>
+      <c r="AD32" s="1"/>
+      <c r="AE32" s="1"/>
+      <c r="AF32" s="1"/>
+      <c r="AG32" s="1"/>
+    </row>
+    <row r="33" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="1"/>
@@ -1001,8 +1563,17 @@
       <c r="T33" s="1"/>
       <c r="U33" s="1"/>
       <c r="V33" s="1"/>
-    </row>
-    <row r="34" spans="4:22" x14ac:dyDescent="0.3">
+      <c r="Y33" s="1"/>
+      <c r="Z33" s="1"/>
+      <c r="AA33" s="1"/>
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="1"/>
+      <c r="AD33" s="1"/>
+      <c r="AE33" s="1"/>
+      <c r="AF33" s="1"/>
+      <c r="AG33" s="1"/>
+    </row>
+    <row r="34" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D34" s="1"/>
       <c r="E34" s="1"/>
       <c r="F34" s="1"/>
@@ -1023,7 +1594,7 @@
       <c r="U34" s="1"/>
       <c r="V34" s="1"/>
     </row>
-    <row r="35" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="35" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D35" s="1"/>
       <c r="E35" s="1"/>
       <c r="F35" s="1"/>
@@ -1044,7 +1615,7 @@
       <c r="U35" s="1"/>
       <c r="V35" s="1"/>
     </row>
-    <row r="36" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="36" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D36" s="1"/>
       <c r="E36" s="1"/>
       <c r="F36" s="1"/>
@@ -1065,7 +1636,7 @@
       <c r="U36" s="1"/>
       <c r="V36" s="1"/>
     </row>
-    <row r="37" spans="4:22" x14ac:dyDescent="0.3">
+    <row r="37" spans="4:33" x14ac:dyDescent="0.3">
       <c r="D37" s="1"/>
       <c r="E37" s="1"/>
       <c r="F37" s="1"/>

</xml_diff>

<commit_message>
feature: Adding a splash screen at startup
</commit_message>
<xml_diff>
--- a/ressources/GPROJ/Tasks.xlsx
+++ b/ressources/GPROJ/Tasks.xlsx
@@ -8,17 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Félisme\Documents\Vector Software Analyzer\vector_software\ressources\GPROJ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAEED8DF-C714-44F2-BF3E-FDDF75C1AB4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706EB929-663E-4BE5-B103-C3DA6FB3B67A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
@@ -28,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="54">
   <si>
     <t>Bug</t>
   </si>
@@ -205,6 +216,17 @@
     <t xml:space="preserve">Récupérer topo
 et calculer l'alti
 au sol </t>
+  </si>
+  <si>
+    <t>Problème
+ Emisphère</t>
+  </si>
+  <si>
+    <t>Faire conversion
+entre NE et SW</t>
+  </si>
+  <si>
+    <t>Remarques d'Eric sur Discord</t>
   </si>
 </sst>
 </file>
@@ -738,15 +760,27 @@
       <c r="AG10" s="1"/>
     </row>
     <row r="11" spans="4:33" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-      <c r="F11" s="1"/>
-      <c r="G11" s="1"/>
-      <c r="H11" s="1"/>
+      <c r="D11" s="5">
+        <v>46150</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G11" s="1">
+        <v>4</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>18</v>
+      </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
-      <c r="L11" s="1"/>
+      <c r="L11" s="1" t="s">
+        <v>53</v>
+      </c>
       <c r="M11" s="4"/>
       <c r="N11" s="5">
         <v>45784</v>

</xml_diff>

<commit_message>
Fix: New polar region return None
</commit_message>
<xml_diff>
--- a/ressources/GPROJ/Tasks.xlsx
+++ b/ressources/GPROJ/Tasks.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
-  <workbookPr/>
+  <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Félisme\Documents\Vector Software Analyzer\vector_software\ressources\GPROJ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706EB929-663E-4BE5-B103-C3DA6FB3B67A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E01D5B-593F-483D-82EA-B13703F6E2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="60">
   <si>
     <t>Bug</t>
   </si>
@@ -87,9 +87,6 @@
   </si>
   <si>
     <t>Date</t>
-  </si>
-  <si>
-    <t>Build trop lourde</t>
   </si>
   <si>
     <t>Changer les imports
@@ -227,6 +224,29 @@
   </si>
   <si>
     <t>Remarques d'Eric sur Discord</t>
+  </si>
+  <si>
+    <t>v0.02</t>
+  </si>
+  <si>
+    <t>Félix</t>
+  </si>
+  <si>
+    <t>DONE</t>
+  </si>
+  <si>
+    <t>à améliorer</t>
+  </si>
+  <si>
+    <t>Build trop
+ lourde</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Crosshair polaire </t>
+  </si>
+  <si>
+    <t>Elles n'apparaissent
+pas tout le temps</t>
   </si>
 </sst>
 </file>
@@ -295,7 +315,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
@@ -306,6 +326,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -586,10 +610,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Feuil1"/>
   <dimension ref="D7:AG37"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
     <col min="6" max="6" width="15.109375" customWidth="1"/>
     <col min="7" max="7" width="13.44140625" customWidth="1"/>
     <col min="8" max="8" width="12.21875" customWidth="1"/>
@@ -605,6 +631,8 @@
     <col min="20" max="20" width="13.77734375" customWidth="1"/>
     <col min="21" max="22" width="13.33203125" customWidth="1"/>
     <col min="25" max="25" width="13.21875" customWidth="1"/>
+    <col min="26" max="26" width="20.77734375" customWidth="1"/>
+    <col min="27" max="27" width="31.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="7" spans="4:33" x14ac:dyDescent="0.3">
@@ -615,7 +643,7 @@
         <v>5</v>
       </c>
       <c r="Y7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="4:33" x14ac:dyDescent="0.3">
@@ -678,7 +706,7 @@
         <v>15</v>
       </c>
       <c r="Z9" s="7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AA9" s="7" t="s">
         <v>6</v>
@@ -702,100 +730,114 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="4:33" ht="115.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="4:33" ht="57.6" x14ac:dyDescent="0.3">
       <c r="D10" s="5">
         <v>46149</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1">
         <v>3</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
-      <c r="N10" s="5">
+      <c r="N10" s="8">
         <v>45784</v>
       </c>
-      <c r="O10" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="P10" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q10" s="1">
+      <c r="O10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q10" s="3">
         <v>3</v>
       </c>
-      <c r="R10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="S10" s="1"/>
-      <c r="T10" s="1"/>
-      <c r="U10" s="1"/>
-      <c r="V10" s="1"/>
+      <c r="R10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="S10" s="8">
+        <v>46153</v>
+      </c>
+      <c r="T10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="U10" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="V10" s="3" t="s">
+        <v>56</v>
+      </c>
       <c r="Y10" s="5">
         <v>46149</v>
       </c>
-      <c r="Z10" s="1" t="s">
+      <c r="Z10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="AA10" s="6" t="s">
         <v>16</v>
-      </c>
-      <c r="AA10" s="6" t="s">
-        <v>17</v>
       </c>
       <c r="AB10" s="1">
         <v>4</v>
       </c>
       <c r="AC10" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AD10" s="1"/>
       <c r="AE10" s="1"/>
       <c r="AF10" s="1"/>
       <c r="AG10" s="1"/>
     </row>
-    <row r="11" spans="4:33" ht="129.6" x14ac:dyDescent="0.3">
-      <c r="D11" s="5">
+    <row r="11" spans="4:33" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="D11" s="8">
         <v>46150</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" s="9" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="G11" s="3">
+        <v>4</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="I11" s="8">
+        <v>46153</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="L11" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="G11" s="1">
-        <v>4</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-      <c r="K11" s="1"/>
-      <c r="L11" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="M11" s="4"/>
       <c r="N11" s="5">
         <v>45784</v>
       </c>
       <c r="O11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="P11" s="6" t="s">
         <v>21</v>
-      </c>
-      <c r="P11" s="6" t="s">
-        <v>22</v>
       </c>
       <c r="Q11" s="1">
         <v>2</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
@@ -805,28 +847,38 @@
         <v>46149</v>
       </c>
       <c r="Z11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="AA11" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="AA11" s="6" t="s">
-        <v>25</v>
       </c>
       <c r="AB11" s="1">
         <v>2</v>
       </c>
       <c r="AC11" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AD11" s="1"/>
       <c r="AE11" s="1"/>
       <c r="AF11" s="1"/>
       <c r="AG11" s="1"/>
     </row>
-    <row r="12" spans="4:33" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
+    <row r="12" spans="4:33" ht="72" x14ac:dyDescent="0.3">
+      <c r="D12" s="5">
+        <v>46154</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="G12" s="1">
+        <v>2</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
@@ -836,16 +888,16 @@
         <v>45784</v>
       </c>
       <c r="O12" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="P12" s="6" t="s">
         <v>26</v>
-      </c>
-      <c r="P12" s="6" t="s">
-        <v>27</v>
       </c>
       <c r="Q12" s="1">
         <v>2</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S12" s="1"/>
       <c r="T12" s="1"/>
@@ -855,23 +907,23 @@
         <v>46149</v>
       </c>
       <c r="Z12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA12" s="6" t="s">
         <v>32</v>
-      </c>
-      <c r="AA12" s="6" t="s">
-        <v>33</v>
       </c>
       <c r="AB12" s="1">
         <v>4</v>
       </c>
       <c r="AC12" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AD12" s="1"/>
       <c r="AE12" s="1"/>
       <c r="AF12" s="1"/>
       <c r="AG12" s="1"/>
     </row>
-    <row r="13" spans="4:33" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="4:33" ht="72" x14ac:dyDescent="0.3">
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
@@ -886,16 +938,16 @@
         <v>45784</v>
       </c>
       <c r="O13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P13" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="P13" s="6" t="s">
-        <v>29</v>
       </c>
       <c r="Q13" s="1">
         <v>2</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S13" s="1"/>
       <c r="T13" s="1"/>
@@ -905,16 +957,16 @@
         <v>46149</v>
       </c>
       <c r="Z13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AA13" s="6" t="s">
         <v>36</v>
-      </c>
-      <c r="AA13" s="6" t="s">
-        <v>37</v>
       </c>
       <c r="AB13" s="1">
         <v>4</v>
       </c>
       <c r="AC13" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AD13" s="1"/>
       <c r="AE13" s="1"/>
@@ -936,16 +988,16 @@
         <v>45784</v>
       </c>
       <c r="O14" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="P14" s="1" t="s">
         <v>30</v>
-      </c>
-      <c r="P14" s="1" t="s">
-        <v>31</v>
       </c>
       <c r="Q14" s="1">
         <v>3</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S14" s="1"/>
       <c r="T14" s="1"/>
@@ -955,16 +1007,16 @@
         <v>46149</v>
       </c>
       <c r="Z14" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="AA14" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="AA14" s="1" t="s">
-        <v>39</v>
       </c>
       <c r="AB14" s="1">
         <v>4</v>
       </c>
       <c r="AC14" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AD14" s="1"/>
       <c r="AE14" s="1"/>
@@ -986,16 +1038,16 @@
         <v>45784</v>
       </c>
       <c r="O15" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="P15" s="6" t="s">
         <v>34</v>
-      </c>
-      <c r="P15" s="6" t="s">
-        <v>35</v>
       </c>
       <c r="Q15" s="1">
         <v>1</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S15" s="1"/>
       <c r="T15" s="1"/>
@@ -1026,14 +1078,14 @@
         <v>45784</v>
       </c>
       <c r="O16" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="P16" s="1"/>
       <c r="Q16" s="1">
         <v>1</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S16" s="1"/>
       <c r="T16" s="1"/>
@@ -1064,16 +1116,16 @@
         <v>45784</v>
       </c>
       <c r="O17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="P17" s="6" t="s">
         <v>41</v>
-      </c>
-      <c r="P17" s="6" t="s">
-        <v>42</v>
       </c>
       <c r="Q17" s="1">
         <v>2</v>
       </c>
       <c r="R17" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S17" s="1"/>
       <c r="T17" s="1"/>
@@ -1104,16 +1156,16 @@
         <v>45784</v>
       </c>
       <c r="O18" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="P18" s="1" t="s">
         <v>44</v>
-      </c>
-      <c r="P18" s="1" t="s">
-        <v>45</v>
       </c>
       <c r="Q18" s="1">
         <v>4</v>
       </c>
       <c r="R18" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S18" s="1"/>
       <c r="T18" s="1"/>
@@ -1144,16 +1196,16 @@
         <v>45784</v>
       </c>
       <c r="O19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="P19" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="P19" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="Q19" s="1">
         <v>2</v>
       </c>
       <c r="R19" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S19" s="1"/>
       <c r="T19" s="1"/>
@@ -1184,14 +1236,14 @@
         <v>45784</v>
       </c>
       <c r="O20" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="P20" s="1"/>
       <c r="Q20" s="1">
         <v>1</v>
       </c>
       <c r="R20" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S20" s="1"/>
       <c r="T20" s="1"/>
@@ -1222,16 +1274,16 @@
         <v>45785</v>
       </c>
       <c r="O21" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="P21" s="6" t="s">
         <v>49</v>
-      </c>
-      <c r="P21" s="6" t="s">
-        <v>50</v>
       </c>
       <c r="Q21" s="1">
         <v>2</v>
       </c>
       <c r="R21" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="S21" s="1"/>
       <c r="T21" s="1"/>

</xml_diff>

<commit_message>
upgrade: Updating readme for Linux , Mac and Windows users
</commit_message>
<xml_diff>
--- a/ressources/GPROJ/Tasks.xlsx
+++ b/ressources/GPROJ/Tasks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Félisme\Documents\Vector Software Analyzer\vector_software\ressources\GPROJ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E01D5B-593F-483D-82EA-B13703F6E2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56020CF3-1124-4902-8563-4CD3DA62CCF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
   <si>
     <t>Bug</t>
   </si>
@@ -247,6 +247,14 @@
   <si>
     <t>Elles n'apparaissent
 pas tout le temps</t>
+  </si>
+  <si>
+    <t>Barbules Skew-T</t>
+  </si>
+  <si>
+    <t>Faire en sorte qu'un nombre constant
+de barbules soit affiché en fonction 
+du zoom</t>
   </si>
 </sst>
 </file>
@@ -1053,11 +1061,21 @@
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
-      <c r="Y15" s="1"/>
-      <c r="Z15" s="1"/>
-      <c r="AA15" s="1"/>
-      <c r="AB15" s="1"/>
-      <c r="AC15" s="1"/>
+      <c r="Y15" s="5">
+        <v>46154</v>
+      </c>
+      <c r="Z15" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AA15" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="AB15" s="1">
+        <v>2</v>
+      </c>
+      <c r="AC15" s="1" t="s">
+        <v>17</v>
+      </c>
       <c r="AD15" s="1"/>
       <c r="AE15" s="1"/>
       <c r="AF15" s="1"/>

</xml_diff>